<commit_message>
updates to schema crate and user guide
</commit_message>
<xml_diff>
--- a/schema/schema-crate/additional-ro-crate-metadata.xlsx
+++ b/schema/schema-crate/additional-ro-crate-metadata.xlsx
@@ -1,25 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10810"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D0F67DD-3591-BD46-B0A3-8C2F575715DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E33A2D-7D28-2E4B-9C0B-D18045DD9AE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RootDataset" sheetId="1" r:id="rId1"/>
     <sheet name="@context" sheetId="2" r:id="rId2"/>
-    <sheet name="File" sheetId="3" r:id="rId3"/>
-    <sheet name="Organization" sheetId="4" r:id="rId4"/>
-    <sheet name="CreativeWork" sheetId="5" r:id="rId5"/>
-    <sheet name="ResourceDescriptor" sheetId="6" r:id="rId6"/>
-    <sheet name="Classes" sheetId="7" r:id="rId7"/>
-    <sheet name="Properties" sheetId="8" r:id="rId8"/>
-    <sheet name="DefinedTermSets" sheetId="9" r:id="rId9"/>
-    <sheet name="DefinedTerms" sheetId="10" r:id="rId10"/>
-    <sheet name="ItemLists" sheetId="11" r:id="rId11"/>
-    <sheet name="ItemInstances" sheetId="12" r:id="rId12"/>
+    <sheet name="Organization" sheetId="4" r:id="rId3"/>
+    <sheet name="CreativeWork" sheetId="5" r:id="rId4"/>
+    <sheet name="ResourceDescriptor" sheetId="6" r:id="rId5"/>
+    <sheet name="Classes" sheetId="7" r:id="rId6"/>
+    <sheet name="Properties" sheetId="8" r:id="rId7"/>
+    <sheet name="DefinedTermSets" sheetId="9" r:id="rId8"/>
+    <sheet name="DefinedTerms" sheetId="10" r:id="rId9"/>
+    <sheet name="ItemLists" sheetId="11" r:id="rId10"/>
+    <sheet name="ItemInstances" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="76">
   <si>
     <t>Name</t>
   </si>
@@ -62,235 +61,211 @@
     <t>name</t>
   </si>
   <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>author</t>
+  </si>
+  <si>
+    <t>license</t>
+  </si>
+  <si>
+    <t>conformsTo</t>
+  </si>
+  <si>
+    <t>hasResource</t>
+  </si>
+  <si>
+    <t>template</t>
+  </si>
+  <si>
+    <t>https://w3id.org/template/terms#</t>
+  </si>
+  <si>
+    <t>https://ror.org/00rqy9422</t>
+  </si>
+  <si>
+    <t>Organization</t>
+  </si>
+  <si>
+    <t>University of Queensland</t>
+  </si>
+  <si>
+    <t>[CreativeWork, Profile]</t>
+  </si>
+  <si>
+    <t>RO-Crate MASP Profile</t>
+  </si>
+  <si>
+    <t>hasRole</t>
+  </si>
+  <si>
+    <t>#hasSpecializedSchema</t>
+  </si>
+  <si>
+    <t>ResourceDescriptor</t>
+  </si>
+  <si>
+    <t>Specialized Schema Terms</t>
+  </si>
+  <si>
+    <t>"http://www.w3.org/ns/dx/prof/role/schema"</t>
+  </si>
+  <si>
+    <t>rdfs:label</t>
+  </si>
+  <si>
+    <t>rdfs:comment</t>
+  </si>
+  <si>
+    <t>rdfs:Class</t>
+  </si>
+  <si>
+    <t>Class Example</t>
+  </si>
+  <si>
+    <t>This is an example of a standard class and its format.</t>
+  </si>
+  <si>
+    <t>template:ItemListClassExample</t>
+  </si>
+  <si>
+    <t>Item List Class Example</t>
+  </si>
+  <si>
+    <t>This is an example of a class to be used as an @type with a list of item instances.</t>
+  </si>
+  <si>
+    <t>domainIncludes</t>
+  </si>
+  <si>
+    <t>rangeIncludes</t>
+  </si>
+  <si>
+    <t>rdf:Property</t>
+  </si>
+  <si>
+    <t>Property Example</t>
+  </si>
+  <si>
+    <t>This is an example of a standard property and its format.</t>
+  </si>
+  <si>
+    <t>"template:ClassExample"</t>
+  </si>
+  <si>
+    <t>"http://schema.org/Text"</t>
+  </si>
+  <si>
+    <t>Defined Term Set Property Example</t>
+  </si>
+  <si>
+    <t>This is an example of a property whose values are expected to be terms from a defined term set.</t>
+  </si>
+  <si>
+    <t>"template:DefinedTermSetExample"</t>
+  </si>
+  <si>
+    <t>Item List Property Example</t>
+  </si>
+  <si>
+    <t>This is an example of a property whose values are expected to be terms from an item list.</t>
+  </si>
+  <si>
+    <t>"#itemListExample"</t>
+  </si>
+  <si>
+    <t>DefinedTermSet</t>
+  </si>
+  <si>
+    <t>Defined Term Set Example</t>
+  </si>
+  <si>
+    <t>This is an example of a defined term set and its format.</t>
+  </si>
+  <si>
+    <t>inDefinedTermSet</t>
+  </si>
+  <si>
+    <t>DefinedTerm</t>
+  </si>
+  <si>
+    <t>Defined Term Example</t>
+  </si>
+  <si>
+    <t>This is an example of a defined term and its format.</t>
+  </si>
+  <si>
+    <t>#itemListExample</t>
+  </si>
+  <si>
+    <t>ItemList</t>
+  </si>
+  <si>
+    <t>Item List Example</t>
+  </si>
+  <si>
+    <t>This is an example of an item list and its format.</t>
+  </si>
+  <si>
+    <t>Item Instance Example</t>
+  </si>
+  <si>
+    <t>This is an example of an item instance and its format.</t>
+  </si>
+  <si>
+    <t>isReverse_hasPart</t>
+  </si>
+  <si>
+    <t>.id</t>
+  </si>
+  <si>
+    <t>ItemListClassExample</t>
+  </si>
+  <si>
+    <t>ClassExample</t>
+  </si>
+  <si>
+    <t>propertyExample</t>
+  </si>
+  <si>
+    <t>definedTermSetPropertyExample</t>
+  </si>
+  <si>
+    <t>itemListPropertyExample</t>
+  </si>
+  <si>
+    <t>DefinedTermSetExample</t>
+  </si>
+  <si>
+    <t>DefinedTermExample</t>
+  </si>
+  <si>
+    <t>itemListExample</t>
+  </si>
+  <si>
+    <t>ItemInstanceExample</t>
+  </si>
+  <si>
+    <t>isReverse_itemListElement</t>
+  </si>
+  <si>
+    <t>https://w3id.org/ro/ro-crate-masp/profile</t>
+  </si>
+  <si>
+    <t>https://www.apache.org/licenses/LICENSE-2.0.html</t>
+  </si>
+  <si>
+    <t>CreativeWork</t>
+  </si>
+  <si>
+    <t>Apache License, Version 2.0</t>
+  </si>
+  <si>
     <t>Template RO-Crate Schema</t>
   </si>
   <si>
-    <t>description</t>
-  </si>
-  <si>
     <t>This is a template for an RO-Crate schema.</t>
-  </si>
-  <si>
-    <t>author</t>
-  </si>
-  <si>
-    <t>license</t>
-  </si>
-  <si>
-    <t>GPL-3.0</t>
-  </si>
-  <si>
-    <t>conformsTo</t>
-  </si>
-  <si>
-    <t>["https://language-research-technology.github.io/ro-crate-masp/profiles/ro-crate-masp/profile-crate/#profile", "https://github.com/Language-Research-Technology/ro-crate-schema-tools/blob/main/profiles/sossplus-profile.md"]</t>
-  </si>
-  <si>
-    <t>hasResource</t>
-  </si>
-  <si>
-    <t>hasPart</t>
-  </si>
-  <si>
-    <t>["schema-documentation.md", "index.html"]</t>
-  </si>
-  <si>
-    <t>template</t>
-  </si>
-  <si>
-    <t>https://w3id.org/template/terms#</t>
-  </si>
-  <si>
-    <t>isPartOf</t>
-  </si>
-  <si>
-    <t>schema-documentation.md</t>
-  </si>
-  <si>
-    <t>File</t>
-  </si>
-  <si>
-    <t>"./"</t>
-  </si>
-  <si>
-    <t>index.html</t>
-  </si>
-  <si>
-    <t>https://ror.org/00rqy9422</t>
-  </si>
-  <si>
-    <t>Organization</t>
-  </si>
-  <si>
-    <t>University of Queensland</t>
-  </si>
-  <si>
-    <t>url</t>
-  </si>
-  <si>
-    <t>https://language-research-technology.github.io/ro-crate-masp/profiles/ro-crate-masp/profile-crate/#profile</t>
-  </si>
-  <si>
-    <t>[CreativeWork, Profile]</t>
-  </si>
-  <si>
-    <t>RO-Crate MASP Profile</t>
-  </si>
-  <si>
-    <t>https://language-research-technology.github.io/ro-crate-masp/profiles/ro-crate-masp/profile-crate/</t>
-  </si>
-  <si>
-    <t>hasRole</t>
-  </si>
-  <si>
-    <t>#hasSpecializedSchema</t>
-  </si>
-  <si>
-    <t>ResourceDescriptor</t>
-  </si>
-  <si>
-    <t>Specialized Schema Terms</t>
-  </si>
-  <si>
-    <t>"http://www.w3.org/ns/dx/prof/role/schema"</t>
-  </si>
-  <si>
-    <t>rdfs:label</t>
-  </si>
-  <si>
-    <t>rdfs:comment</t>
-  </si>
-  <si>
-    <t>rdfs:Class</t>
-  </si>
-  <si>
-    <t>Class Example</t>
-  </si>
-  <si>
-    <t>This is an example of a standard class and its format.</t>
-  </si>
-  <si>
-    <t>template:ItemListClassExample</t>
-  </si>
-  <si>
-    <t>Item List Class Example</t>
-  </si>
-  <si>
-    <t>This is an example of a class to be used as an @type with a list of item instances.</t>
-  </si>
-  <si>
-    <t>domainIncludes</t>
-  </si>
-  <si>
-    <t>rangeIncludes</t>
-  </si>
-  <si>
-    <t>rdf:Property</t>
-  </si>
-  <si>
-    <t>Property Example</t>
-  </si>
-  <si>
-    <t>This is an example of a standard property and its format.</t>
-  </si>
-  <si>
-    <t>"template:ClassExample"</t>
-  </si>
-  <si>
-    <t>"http://schema.org/Text"</t>
-  </si>
-  <si>
-    <t>Defined Term Set Property Example</t>
-  </si>
-  <si>
-    <t>This is an example of a property whose values are expected to be terms from a defined term set.</t>
-  </si>
-  <si>
-    <t>"template:DefinedTermSetExample"</t>
-  </si>
-  <si>
-    <t>Item List Property Example</t>
-  </si>
-  <si>
-    <t>This is an example of a property whose values are expected to be terms from an item list.</t>
-  </si>
-  <si>
-    <t>"#itemListExample"</t>
-  </si>
-  <si>
-    <t>DefinedTermSet</t>
-  </si>
-  <si>
-    <t>Defined Term Set Example</t>
-  </si>
-  <si>
-    <t>This is an example of a defined term set and its format.</t>
-  </si>
-  <si>
-    <t>inDefinedTermSet</t>
-  </si>
-  <si>
-    <t>DefinedTerm</t>
-  </si>
-  <si>
-    <t>Defined Term Example</t>
-  </si>
-  <si>
-    <t>This is an example of a defined term and its format.</t>
-  </si>
-  <si>
-    <t>#itemListExample</t>
-  </si>
-  <si>
-    <t>ItemList</t>
-  </si>
-  <si>
-    <t>Item List Example</t>
-  </si>
-  <si>
-    <t>This is an example of an item list and its format.</t>
-  </si>
-  <si>
-    <t>Item Instance Example</t>
-  </si>
-  <si>
-    <t>This is an example of an item instance and its format.</t>
-  </si>
-  <si>
-    <t>isReverse_hasPart</t>
-  </si>
-  <si>
-    <t>.id</t>
-  </si>
-  <si>
-    <t>ItemListClassExample</t>
-  </si>
-  <si>
-    <t>ClassExample</t>
-  </si>
-  <si>
-    <t>propertyExample</t>
-  </si>
-  <si>
-    <t>definedTermSetPropertyExample</t>
-  </si>
-  <si>
-    <t>itemListPropertyExample</t>
-  </si>
-  <si>
-    <t>DefinedTermSetExample</t>
-  </si>
-  <si>
-    <t>DefinedTermExample</t>
-  </si>
-  <si>
-    <t>itemListExample</t>
-  </si>
-  <si>
-    <t>ItemInstanceExample</t>
-  </si>
-  <si>
-    <t>isReverse_itemListElement</t>
   </si>
 </sst>
 </file>
@@ -317,18 +292,12 @@
       <name val="Aptos"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.79998168889431442"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -349,13 +318,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -695,7 +662,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.1640625" style="2" bestFit="1" customWidth="1"/>
@@ -732,20 +699,20 @@
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>7</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>9</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="str">
         <f>"""" &amp; Organization!A2 &amp; """"</f>
@@ -754,35 +721,29 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>12</v>
+        <v>9</v>
+      </c>
+      <c r="B7" s="1" t="str">
+        <f>"""" &amp; CreativeWork!A3 &amp; """"</f>
+        <v>"https://www.apache.org/licenses/LICENSE-2.0.html"</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>14</v>
+        <v>10</v>
+      </c>
+      <c r="B8" s="1" t="str">
+        <f>"""" &amp; CreativeWork!A2 &amp; """"</f>
+        <v>"https://w3id.org/ro/ro-crate-masp/profile"</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="B9" s="1" t="str">
         <f>"""" &amp; ResourceDescriptor!A2 &amp; """"</f>
         <v>"#hasSpecializedSchema"</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -792,83 +753,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="33.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="53.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.83203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="str">
-        <f>'@context'!$A$2 &amp; ":" &amp; B2</f>
-        <v>template:DefinedTermExample</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F2" s="1" t="str">
-        <f>A2</f>
-        <v>template:DefinedTermExample</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="H2" s="1" t="str">
-        <f>ResourceDescriptor!$A$2</f>
-        <v>#hasSpecializedSchema</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -886,7 +770,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -895,7 +779,7 @@
         <v>6</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -904,16 +788,16 @@
         <v>#itemListExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>68</v>
+        <v>54</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>69</v>
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -922,7 +806,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -943,7 +827,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -952,16 +836,16 @@
         <v>6</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -970,23 +854,23 @@
         <v>template:ItemInstanceExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="F2" s="1" t="str">
         <f>A2</f>
         <v>template:ItemInstanceExample</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="H2" s="1" t="str">
         <f>ResourceDescriptor!$A$2</f>
@@ -1019,10 +903,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>19</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1032,66 +916,6 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="30.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="30.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.83203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B3" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>23</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -1115,13 +939,64 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>27</v>
+        <v>16</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="A1:C3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="55.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="29.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1131,52 +1006,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="114.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="106.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.83203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -1199,21 +1028,21 @@
         <v>6</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1222,7 +1051,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -1243,7 +1072,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -1252,16 +1081,16 @@
         <v>6</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1270,16 +1099,16 @@
         <v>template:ClassExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>41</v>
+        <v>27</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="F2" s="1" t="str">
         <f>A2</f>
@@ -1300,16 +1129,16 @@
         <v>template:ItemListClassExample</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>74</v>
+        <v>60</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>44</v>
+        <v>30</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="F3" s="1" t="str">
         <f>A3</f>
@@ -1330,7 +1159,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -1353,7 +1182,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -1362,22 +1191,22 @@
         <v>6</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -1386,22 +1215,22 @@
         <v>template:propertyExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="H2" s="1" t="str">
         <f>D2</f>
@@ -1422,22 +1251,22 @@
         <v>template:definedTermSetPropertyExample</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
       <c r="H3" s="1" t="str">
         <f t="shared" ref="H3:H4" si="0">D3</f>
@@ -1458,22 +1287,22 @@
         <v>template:itemListPropertyExample</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>56</v>
+        <v>42</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="H4" s="1" t="str">
         <f t="shared" si="0"/>
@@ -1494,7 +1323,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -1514,7 +1343,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -1523,13 +1352,13 @@
         <v>6</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1538,22 +1367,99 @@
         <v>template:DefinedTermSetExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>60</v>
+        <v>46</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="F2" s="1" t="str">
         <f>A2</f>
         <v>template:DefinedTermSetExample</v>
       </c>
       <c r="G2" s="1" t="str">
+        <f>ResourceDescriptor!$A$2</f>
+        <v>#hasSpecializedSchema</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="33.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="53.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="str">
+        <f>'@context'!$A$2 &amp; ":" &amp; B2</f>
+        <v>template:DefinedTermExample</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="1" t="str">
+        <f>A2</f>
+        <v>template:DefinedTermExample</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="H2" s="1" t="str">
         <f>ResourceDescriptor!$A$2</f>
         <v>#hasSpecializedSchema</v>
       </c>

</xml_diff>

<commit_message>
item list element and link updates
</commit_message>
<xml_diff>
--- a/schema/schema-crate/additional-ro-crate-metadata.xlsx
+++ b/schema/schema-crate/additional-ro-crate-metadata.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10810"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9E33A2D-7D28-2E4B-9C0B-D18045DD9AE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E23F0763-8D95-FB47-BC04-1596A71AF3E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="26400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4500" yWindow="1200" windowWidth="25460" windowHeight="18440" firstSheet="1" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RootDataset" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,7 @@
     <sheet name="DefinedTermSets" sheetId="9" r:id="rId8"/>
     <sheet name="DefinedTerms" sheetId="10" r:id="rId9"/>
     <sheet name="ItemLists" sheetId="11" r:id="rId10"/>
-    <sheet name="ItemInstances" sheetId="12" r:id="rId11"/>
+    <sheet name="ItemListElements" sheetId="12" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -208,12 +208,6 @@
     <t>This is an example of an item list and its format.</t>
   </si>
   <si>
-    <t>Item Instance Example</t>
-  </si>
-  <si>
-    <t>This is an example of an item instance and its format.</t>
-  </si>
-  <si>
     <t>isReverse_hasPart</t>
   </si>
   <si>
@@ -244,9 +238,6 @@
     <t>itemListExample</t>
   </si>
   <si>
-    <t>ItemInstanceExample</t>
-  </si>
-  <si>
     <t>isReverse_itemListElement</t>
   </si>
   <si>
@@ -266,6 +257,15 @@
   </si>
   <si>
     <t>This is a template for an RO-Crate schema.</t>
+  </si>
+  <si>
+    <t>ItemListElementExample</t>
+  </si>
+  <si>
+    <t>This is an example of an item list element and its format.</t>
+  </si>
+  <si>
+    <t>Item List Element Example</t>
   </si>
 </sst>
 </file>
@@ -699,7 +699,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -707,7 +707,7 @@
         <v>7</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -770,7 +770,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -788,7 +788,7 @@
         <v>#itemListExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>53</v>
@@ -811,12 +811,12 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="33.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="37.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="27.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="55.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="59.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="30.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="27.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="8.83203125" style="1"/>
@@ -827,7 +827,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -842,32 +842,32 @@
         <v>24</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="str">
         <f>'@context'!$A$2 &amp; ":" &amp; B2</f>
-        <v>template:ItemInstanceExample</v>
+        <v>template:ItemListElementExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>29</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>57</v>
+        <v>74</v>
       </c>
       <c r="F2" s="1" t="str">
         <f>A2</f>
-        <v>template:ItemInstanceExample</v>
+        <v>template:ItemListElementExample</v>
       </c>
       <c r="G2" s="3" t="s">
         <v>52</v>
@@ -979,7 +979,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>17</v>
@@ -990,13 +990,13 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1072,7 +1072,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -1090,7 +1090,7 @@
         <v>25</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1099,7 +1099,7 @@
         <v>template:ClassExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>26</v>
@@ -1129,7 +1129,7 @@
         <v>template:ItemListClassExample</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>26</v>
@@ -1182,7 +1182,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -1206,7 +1206,7 @@
         <v>25</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -1215,7 +1215,7 @@
         <v>template:propertyExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>34</v>
@@ -1251,7 +1251,7 @@
         <v>template:definedTermSetPropertyExample</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>34</v>
@@ -1287,7 +1287,7 @@
         <v>template:itemListPropertyExample</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>34</v>
@@ -1343,7 +1343,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -1358,7 +1358,7 @@
         <v>24</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -1367,7 +1367,7 @@
         <v>template:DefinedTermSetExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>45</v>
@@ -1414,7 +1414,7 @@
         <v>2</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>4</v>
@@ -1432,7 +1432,7 @@
         <v>48</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -1441,7 +1441,7 @@
         <v>template:DefinedTermExample</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>49</v>

</xml_diff>

<commit_message>
schema template and guide updates
</commit_message>
<xml_diff>
--- a/schema/schema-crate/additional-ro-crate-metadata.xlsx
+++ b/schema/schema-crate/additional-ro-crate-metadata.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10817"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10821"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE8F47C-53E9-174B-AA12-7CA814053B01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7691B873-4DB6-2E47-8054-F350FC290032}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4500" yWindow="1200" windowWidth="25460" windowHeight="18440" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="640" yWindow="600" windowWidth="25460" windowHeight="18440" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="RootDataset" sheetId="1" r:id="rId1"/>
@@ -13,12 +13,13 @@
     <sheet name="Organization" sheetId="4" r:id="rId3"/>
     <sheet name="CreativeWork" sheetId="5" r:id="rId4"/>
     <sheet name="ResourceDescriptor" sheetId="6" r:id="rId5"/>
-    <sheet name="Classes" sheetId="7" r:id="rId6"/>
-    <sheet name="Properties" sheetId="8" r:id="rId7"/>
-    <sheet name="DefinedTermSets" sheetId="9" r:id="rId8"/>
-    <sheet name="DefinedTerms" sheetId="10" r:id="rId9"/>
-    <sheet name="ItemLists" sheetId="11" r:id="rId10"/>
-    <sheet name="ItemListElements" sheetId="12" r:id="rId11"/>
+    <sheet name="Schema" sheetId="13" r:id="rId6"/>
+    <sheet name="Classes" sheetId="7" r:id="rId7"/>
+    <sheet name="Properties" sheetId="8" r:id="rId8"/>
+    <sheet name="DefinedTermSets" sheetId="9" r:id="rId9"/>
+    <sheet name="DefinedTerms" sheetId="10" r:id="rId10"/>
+    <sheet name="ItemLists" sheetId="11" r:id="rId11"/>
+    <sheet name="ItemListElements" sheetId="12" r:id="rId12"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="80">
   <si>
     <t>Name</t>
   </si>
@@ -265,7 +266,19 @@
     <t>Item List Element Example</t>
   </si>
   <si>
-    <t>arcp://name,template-schema/terms#</t>
+    <t>arcp://name,template/terms#</t>
+  </si>
+  <si>
+    <t>http://www.w3.org/ns/dx/prof/role/schema</t>
+  </si>
+  <si>
+    <t>DefinedTerm, ResourceRole]</t>
+  </si>
+  <si>
+    <t>Schema</t>
+  </si>
+  <si>
+    <t>Machine-readable structural descriptions of data defined by the profile</t>
   </si>
 </sst>
 </file>
@@ -318,11 +331,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -666,7 +681,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.1640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="242.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="57.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
@@ -753,6 +768,83 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
+  <dimension ref="A1:H2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="33.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="53.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="33.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="38.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="27.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="str">
+        <f>'@context'!$A$2 &amp; ":" &amp; B2</f>
+        <v>template:DefinedTermExample</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="F2" s="1" t="str">
+        <f>A2</f>
+        <v>template:DefinedTermExample</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H2" s="1" t="str">
+        <f>ResourceDescriptor!$A$2</f>
+        <v>#hasSpecializedSchema</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -806,7 +898,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -889,7 +981,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="32.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
@@ -1041,7 +1133,7 @@
       <c r="C2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="5" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1052,6 +1144,52 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{501760DB-06F6-5040-87D7-73A396868E3D}">
+  <dimension ref="A1:D2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="46.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="74.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -1159,7 +1297,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -1323,7 +1461,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:G2"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
@@ -1391,81 +1529,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="33.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="23.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="24.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="53.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="33.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="38.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="27.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="16384" width="8.83203125" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="str">
-        <f>'@context'!$A$2 &amp; ":" &amp; B2</f>
-        <v>template:DefinedTermExample</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="F2" s="1" t="str">
-        <f>A2</f>
-        <v>template:DefinedTermExample</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H2" s="1" t="str">
-        <f>ResourceDescriptor!$A$2</f>
-        <v>#hasSpecializedSchema</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-</worksheet>
 </file>
</xml_diff>